<commit_message>
v1.1 - edit cat
</commit_message>
<xml_diff>
--- a/MiAtlas-Database-Starter.xlsx
+++ b/MiAtlas-Database-Starter.xlsx
@@ -544,9 +544,7 @@
           <t>2,865 m · the legendary dinosaur-spine ridge · trekked together 🤝</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
       <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -580,9 +578,7 @@
           <t>2,881 m · 'the Vietnamese Everest', one of the toughest treks · trekked together 🤝</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
       <c r="I3" s="2" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -616,9 +612,7 @@
           <t>3,143 m · the Roof of Indochina, Vietnam's highest</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
       <c r="I4" s="2" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -652,9 +646,7 @@
           <t>3,083 m · 2nd highest · remote border peak, multi-day</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
       <c r="I5" s="2" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -688,9 +680,7 @@
           <t>3,049 m · rhododendron forests in spring</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
       <c r="I6" s="2" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -724,9 +714,7 @@
           <t>3,046 m · famous 'heaven's gate' cloud sea</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
       <c r="I7" s="2" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -760,9 +748,7 @@
           <t>3,012 m · Lai Châu border, French stele on summit</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
       <c r="I8" s="2" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -796,9 +782,7 @@
           <t>2,979 m · purple Chi Pâu flower season (Oct)</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
       <c r="I9" s="2" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -832,9 +816,7 @@
           <t>2,965 m · the 'waterfall in the clouds' trek</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
       <c r="I10" s="2" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -868,9 +850,7 @@
           <t>2,860 m · the 'lonely peak', best beginner cloud-hunt</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
       <c r="I11" s="2" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -904,9 +884,7 @@
           <t>2,402 m · Hà Giang's shimmering cloud throne</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr"/>
       <c r="I12" s="2" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -940,9 +918,7 @@
           <t>Easternmost point of mainland Vietnam · first sunrise</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr"/>
       <c r="I13" s="2" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -976,9 +952,7 @@
           <t>Turquoise coves &amp; windy cliffs</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr"/>
       <c r="I14" s="2" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1012,9 +986,7 @@
           <t>Volcanic island, garlic fields, Hang Câu</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
       <c r="I15" s="2" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1048,9 +1020,7 @@
           <t>Marine reserve, snorkelling, no plastic</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr"/>
       <c r="I16" s="2" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1084,9 +1054,7 @@
           <t>Off-grid island, windmills &amp; wild coves</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr"/>
       <c r="I17" s="2" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1120,9 +1088,7 @@
           <t>Lobster islands, clear water, backpacker fave</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
       <c r="I18" s="2" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1156,9 +1122,7 @@
           <t>21 islands, untouched fishing-village vibe</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr"/>
       <c r="I19" s="2" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1192,9 +1156,7 @@
           <t>Wild beach below the runway, sea turtles</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr"/>
       <c r="I20" s="2" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1228,9 +1190,7 @@
           <t>Northern island, white sand &amp; clear sea</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr"/>
       <c r="I21" s="2" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1264,9 +1224,7 @@
           <t>Quieter, wilder cousin of Hạ Long Bay</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr"/>
       <c r="I22" s="2" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1300,9 +1258,7 @@
           <t>The legendary 3–4 day northern motorbike loop</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr"/>
       <c r="I23" s="2" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1336,9 +1292,7 @@
           <t>'King of passes' above the Nho Quế river canyon</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr"/>
       <c r="I24" s="2" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1372,9 +1326,7 @@
           <t>Longest pass in VN, Sa Pa ↔ Lai Châu</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr"/>
       <c r="I25" s="2" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1408,9 +1360,7 @@
           <t>Pass over the golden rice terraces</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
       <c r="I26" s="2" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1444,9 +1394,7 @@
           <t>Sơn La ↔ Điện Biên, one of the 'four great passes'</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr"/>
       <c r="I27" s="2" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1480,9 +1428,7 @@
           <t>Ocean cliff pass, Huế ↔ Đà Nẵng</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
       <c r="I28" s="2" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1516,9 +1462,7 @@
           <t>Northeast loop ending at the giant border waterfall</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr"/>
       <c r="I29" s="2" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1552,9 +1496,7 @@
           <t>Golden terraced rice fields (Sept–Oct)</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr"/>
       <c r="I30" s="2" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1588,9 +1530,7 @@
           <t>Trekking hub of the northwest</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr"/>
       <c r="I31" s="2" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1624,9 +1564,7 @@
           <t>World's largest cave &amp; karst wonderland</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr"/>
       <c r="I32" s="2" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1660,9 +1598,7 @@
           <t>UNESCO Geopark on the Hà Giang loop</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr"/>
       <c r="I33" s="2" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1696,9 +1632,7 @@
           <t>'Halong on land', river caves &amp; karst</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr"/>
       <c r="I34" s="2" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="2">
@@ -1735,7 +1669,6 @@
       <c r="B1" s="2" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
       <c r="B2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
@@ -1795,7 +1728,6 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr"/>
       <c r="B8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
@@ -1838,7 +1770,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Một trong: peak / sea / loop / highlight.</t>
+          <t>4 loại sẵn: peak / sea / loop / highlight. Có thể tự gõ loại MỚI (vd food, waterfall, camp) — app tự nhận, hiện icon 📍. Gõ nhất quán một cách viết cho cùng loại.</t>
         </is>
       </c>
     </row>
@@ -1931,7 +1863,6 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr"/>
       <c r="B21" s="2" t="inlineStr">
         <is>
           <t>Đừng sửa tay sheet trong lúc app đang mở &amp; đang đẩy dữ liệu — sửa một bên rồi để bên kia kéo về.</t>

</xml_diff>